<commit_message>
Άδειες με βάση τον πίνακα του m365maps: Entra Suite και Governance στο E7, device inventory στο Defender for Endpoint Plan 2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M4snhbgdNH6z5QRgt779xt
</commit_message>
<xml_diff>
--- a/static/downloads/iso-27001-2022-annex-a-microsoft-365-checklist.xlsx
+++ b/static/downloads/iso-27001-2022-annex-a-microsoft-365-checklist.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="864" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="565">
   <si>
     <t xml:space="preserve">ISO/IEC 27001:2022 Annex A και Microsoft 365: checklist</t>
   </si>
@@ -513,7 +513,7 @@
     <t xml:space="preserve">Entra ID: audit logs δημιουργίας και απενεργοποίησης λογαριασμών, ιστορικό lifecycle workflows.</t>
   </si>
   <si>
-    <t xml:space="preserve">Microsoft Entra ID Governance (lifecycle workflows)</t>
+    <t xml:space="preserve">Microsoft Entra ID Governance (lifecycle workflows· πρόσθετο, περιλαμβάνεται στο Microsoft 365 E7)</t>
   </si>
   <si>
     <t xml:space="preserve">https://thecybersec.gr/posts/global-secure-access/global-secure-access-meros-5-conditional-access/
@@ -1035,7 +1035,7 @@
     <t xml:space="preserve">Entra ID: πολιτικές Conditional Access. Intune: αναφορές συμμόρφωσης συσκευών.</t>
   </si>
   <si>
-    <t xml:space="preserve">Microsoft Entra Private Access</t>
+    <t xml:space="preserve">Microsoft Entra Private Access (Microsoft Entra Suite ή standalone· περιλαμβάνεται στο Microsoft 365 E7)</t>
   </si>
   <si>
     <t xml:space="preserve">13, 19</t>
@@ -1265,6 +1265,9 @@
     <t xml:space="preserve">Intune: αναφορές συμμόρφωσης. Defender for Endpoint: device inventory με κατάσταση onboarding.</t>
   </si>
   <si>
+    <t xml:space="preserve">Microsoft Defender for Endpoint Plan 2 (Microsoft 365 E5 ή αντίστοιχο) για το device inventory</t>
+  </si>
+  <si>
     <t xml:space="preserve">14, 20</t>
   </si>
   <si>
@@ -1457,7 +1460,7 @@
     <t xml:space="preserve">Purview: DLP policies, alerts και Activity explorer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Microsoft 365 E5 (Endpoint DLP, Teams DLP, Network Data Security), Microsoft Entra Internet Access (Network Data Security)</t>
+    <t xml:space="preserve">Microsoft 365 E5 (Endpoint DLP, Teams DLP, Network Data Security), Microsoft Entra Internet Access (Network Data Security· Microsoft Entra Suite, standalone ή Microsoft 365 E7)</t>
   </si>
   <si>
     <t xml:space="preserve">A.8.13</t>
@@ -1595,7 +1598,7 @@
     <t xml:space="preserve">Ρυθμίσεις firewall. Intune: πολιτικές Windows Firewall.</t>
   </si>
   <si>
-    <t xml:space="preserve">Microsoft Entra Internet Access, Microsoft Entra Private Access</t>
+    <t xml:space="preserve">Microsoft Entra Internet Access (Microsoft Entra Suite ή standalone· περιλαμβάνεται στο Microsoft 365 E7), Microsoft Entra Private Access (Microsoft Entra Suite ή standalone· περιλαμβάνεται στο Microsoft 365 E7)</t>
   </si>
   <si>
     <t xml:space="preserve">19</t>
@@ -1651,7 +1654,7 @@
     <t xml:space="preserve">Defender portal: web content filtering policies και web protection report.</t>
   </si>
   <si>
-    <t xml:space="preserve">Microsoft Entra Internet Access</t>
+    <t xml:space="preserve">Microsoft Entra Internet Access (Microsoft Entra Suite ή standalone· περιλαμβάνεται στο Microsoft 365 E7)</t>
   </si>
   <si>
     <t xml:space="preserve">19, 20</t>
@@ -4914,13 +4917,15 @@
       <c r="H61" s="8" t="s">
         <v>380</v>
       </c>
-      <c r="I61" s="8"/>
+      <c r="I61" s="8" t="s">
+        <v>381</v>
+      </c>
       <c r="J61" s="8"/>
       <c r="K61" s="7" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="L61" s="8" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="M61" s="9"/>
       <c r="N61" s="10"/>
@@ -4930,7 +4935,7 @@
     </row>
     <row r="62" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B62" s="7" t="n">
         <v>8</v>
@@ -4940,16 +4945,16 @@
       </c>
       <c r="D62" s="8"/>
       <c r="E62" s="8" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F62" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G62" s="8" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="H62" s="8" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="I62" s="8" t="s">
         <v>79</v>
@@ -4969,7 +4974,7 @@
     </row>
     <row r="63" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B63" s="7" t="n">
         <v>8</v>
@@ -4979,16 +4984,16 @@
       </c>
       <c r="D63" s="8"/>
       <c r="E63" s="8" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F63" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="H63" s="8" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="I63" s="8"/>
       <c r="J63" s="8"/>
@@ -4996,7 +5001,7 @@
         <v>148</v>
       </c>
       <c r="L63" s="8" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="M63" s="9"/>
       <c r="N63" s="10"/>
@@ -5006,7 +5011,7 @@
     </row>
     <row r="64" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B64" s="7" t="n">
         <v>8</v>
@@ -5016,19 +5021,19 @@
       </c>
       <c r="D64" s="8"/>
       <c r="E64" s="8" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F64" s="8" t="s">
         <v>44</v>
       </c>
       <c r="G64" s="8" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="H64" s="8" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="I64" s="8" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="J64" s="8"/>
       <c r="K64" s="7" t="s">
@@ -5043,7 +5048,7 @@
     </row>
     <row r="65" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B65" s="7" t="n">
         <v>8</v>
@@ -5053,16 +5058,16 @@
       </c>
       <c r="D65" s="8"/>
       <c r="E65" s="8" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F65" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="H65" s="8" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="I65" s="8"/>
       <c r="J65" s="8"/>
@@ -5080,7 +5085,7 @@
     </row>
     <row r="66" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B66" s="7" t="n">
         <v>8</v>
@@ -5090,20 +5095,20 @@
       </c>
       <c r="D66" s="8"/>
       <c r="E66" s="8" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F66" s="8" t="s">
         <v>44</v>
       </c>
       <c r="G66" s="8" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="H66" s="8" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="I66" s="8"/>
       <c r="J66" s="8" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="K66" s="7"/>
       <c r="L66" s="8"/>
@@ -5115,7 +5120,7 @@
     </row>
     <row r="67" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B67" s="7" t="n">
         <v>8</v>
@@ -5125,26 +5130,26 @@
       </c>
       <c r="D67" s="8"/>
       <c r="E67" s="8" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F67" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="H67" s="8" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="J67" s="8"/>
       <c r="K67" s="7" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="L67" s="8" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="M67" s="9"/>
       <c r="N67" s="10"/>
@@ -5154,7 +5159,7 @@
     </row>
     <row r="68" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B68" s="7" t="n">
         <v>8</v>
@@ -5164,19 +5169,19 @@
       </c>
       <c r="D68" s="8"/>
       <c r="E68" s="8" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F68" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G68" s="8" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="H68" s="8" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="I68" s="8" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="J68" s="8"/>
       <c r="K68" s="7" t="s">
@@ -5193,7 +5198,7 @@
     </row>
     <row r="69" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B69" s="7" t="n">
         <v>8</v>
@@ -5205,26 +5210,26 @@
         <v>98</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F69" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="H69" s="8" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="I69" s="8" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="J69" s="8"/>
       <c r="K69" s="7" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="L69" s="8" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="M69" s="9"/>
       <c r="N69" s="10"/>
@@ -5234,7 +5239,7 @@
     </row>
     <row r="70" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B70" s="7" t="n">
         <v>8</v>
@@ -5246,19 +5251,19 @@
         <v>98</v>
       </c>
       <c r="E70" s="8" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F70" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G70" s="8" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="H70" s="8" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="I70" s="8" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="J70" s="8"/>
       <c r="K70" s="7" t="s">
@@ -5275,7 +5280,7 @@
     </row>
     <row r="71" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B71" s="7" t="n">
         <v>8</v>
@@ -5287,19 +5292,19 @@
         <v>98</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F71" s="8" t="s">
         <v>44</v>
       </c>
       <c r="G71" s="8" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H71" s="8" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="J71" s="8"/>
       <c r="K71" s="7"/>
@@ -5310,9 +5315,9 @@
       <c r="P71" s="11"/>
       <c r="Q71" s="10"/>
     </row>
-    <row r="72" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B72" s="7" t="n">
         <v>8</v>
@@ -5324,19 +5329,19 @@
         <v>98</v>
       </c>
       <c r="E72" s="8" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F72" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G72" s="8" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H72" s="8" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="I72" s="8" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="J72" s="8"/>
       <c r="K72" s="7" t="s">
@@ -5353,7 +5358,7 @@
     </row>
     <row r="73" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B73" s="7" t="n">
         <v>8</v>
@@ -5363,19 +5368,19 @@
       </c>
       <c r="D73" s="8"/>
       <c r="E73" s="8" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F73" s="8" t="s">
         <v>42</v>
       </c>
       <c r="G73" s="8" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="H73" s="8" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="I73" s="8" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="J73" s="8" t="s">
         <v>238</v>
@@ -5392,7 +5397,7 @@
     </row>
     <row r="74" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B74" s="7" t="n">
         <v>8</v>
@@ -5402,22 +5407,22 @@
       </c>
       <c r="D74" s="8"/>
       <c r="E74" s="8" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F74" s="8" t="s">
         <v>44</v>
       </c>
       <c r="G74" s="8" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="H74" s="8" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="I74" s="8" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J74" s="8" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="K74" s="7" t="s">
         <v>232</v>
@@ -5431,7 +5436,7 @@
     </row>
     <row r="75" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B75" s="7" t="n">
         <v>8</v>
@@ -5441,22 +5446,22 @@
       </c>
       <c r="D75" s="8"/>
       <c r="E75" s="8" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F75" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G75" s="8" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="H75" s="8" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="I75" s="8" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="J75" s="8" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="K75" s="7" t="s">
         <v>91</v>
@@ -5472,7 +5477,7 @@
     </row>
     <row r="76" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B76" s="7" t="n">
         <v>8</v>
@@ -5484,19 +5489,19 @@
         <v>98</v>
       </c>
       <c r="E76" s="8" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="F76" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G76" s="8" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="H76" s="8" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="I76" s="8" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="J76" s="8"/>
       <c r="K76" s="7" t="s">
@@ -5513,7 +5518,7 @@
     </row>
     <row r="77" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B77" s="7" t="n">
         <v>8</v>
@@ -5523,16 +5528,16 @@
       </c>
       <c r="D77" s="8"/>
       <c r="E77" s="8" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F77" s="8" t="s">
         <v>44</v>
       </c>
       <c r="G77" s="8" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="H77" s="8" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="I77" s="8"/>
       <c r="J77" s="8"/>
@@ -5546,7 +5551,7 @@
     </row>
     <row r="78" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B78" s="7" t="n">
         <v>8</v>
@@ -5556,26 +5561,26 @@
       </c>
       <c r="D78" s="8"/>
       <c r="E78" s="8" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F78" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G78" s="8" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="H78" s="8" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="I78" s="8" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="J78" s="8"/>
       <c r="K78" s="7" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="L78" s="8" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="M78" s="9"/>
       <c r="N78" s="10"/>
@@ -5585,7 +5590,7 @@
     </row>
     <row r="79" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="B79" s="7" t="n">
         <v>8</v>
@@ -5595,24 +5600,24 @@
       </c>
       <c r="D79" s="8"/>
       <c r="E79" s="8" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F79" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G79" s="8" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="H79" s="8" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="I79" s="8"/>
       <c r="J79" s="8"/>
       <c r="K79" s="7" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="L79" s="8" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="M79" s="9"/>
       <c r="N79" s="10"/>
@@ -5620,9 +5625,9 @@
       <c r="P79" s="11"/>
       <c r="Q79" s="10"/>
     </row>
-    <row r="80" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="B80" s="7" t="n">
         <v>8</v>
@@ -5632,26 +5637,26 @@
       </c>
       <c r="D80" s="8"/>
       <c r="E80" s="8" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F80" s="8" t="s">
         <v>42</v>
       </c>
       <c r="G80" s="8" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="H80" s="8" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="I80" s="8" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J80" s="8"/>
       <c r="K80" s="7" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="L80" s="8" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="M80" s="9"/>
       <c r="N80" s="10"/>
@@ -5659,9 +5664,9 @@
       <c r="P80" s="11"/>
       <c r="Q80" s="10"/>
     </row>
-    <row r="81" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B81" s="7" t="n">
         <v>8</v>
@@ -5671,26 +5676,26 @@
       </c>
       <c r="D81" s="8"/>
       <c r="E81" s="8" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="F81" s="8" t="s">
         <v>42</v>
       </c>
       <c r="G81" s="8" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="H81" s="8" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="I81" s="8" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J81" s="8"/>
       <c r="K81" s="7" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="L81" s="8" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="M81" s="9"/>
       <c r="N81" s="10"/>
@@ -5700,7 +5705,7 @@
     </row>
     <row r="82" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="B82" s="7" t="n">
         <v>8</v>
@@ -5710,26 +5715,26 @@
       </c>
       <c r="D82" s="8"/>
       <c r="E82" s="8" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F82" s="8" t="s">
         <v>42</v>
       </c>
       <c r="G82" s="8" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="H82" s="8" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="I82" s="8" t="s">
         <v>311</v>
       </c>
       <c r="J82" s="8"/>
       <c r="K82" s="7" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="L82" s="8" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="M82" s="9"/>
       <c r="N82" s="10"/>
@@ -5739,7 +5744,7 @@
     </row>
     <row r="83" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B83" s="7" t="n">
         <v>8</v>
@@ -5751,26 +5756,26 @@
         <v>98</v>
       </c>
       <c r="E83" s="8" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F83" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G83" s="8" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="H83" s="8" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="I83" s="8" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="J83" s="8"/>
       <c r="K83" s="7" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="L83" s="8" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="M83" s="9"/>
       <c r="N83" s="10"/>
@@ -5780,7 +5785,7 @@
     </row>
     <row r="84" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B84" s="7" t="n">
         <v>8</v>
@@ -5790,28 +5795,28 @@
       </c>
       <c r="D84" s="8"/>
       <c r="E84" s="8" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F84" s="8" t="s">
         <v>40</v>
       </c>
       <c r="G84" s="8" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H84" s="8" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="I84" s="8" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="J84" s="8" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="K84" s="7" t="s">
         <v>141</v>
       </c>
       <c r="L84" s="8" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="M84" s="9"/>
       <c r="N84" s="10"/>
@@ -5821,7 +5826,7 @@
     </row>
     <row r="85" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B85" s="7" t="n">
         <v>8</v>
@@ -5831,26 +5836,26 @@
       </c>
       <c r="D85" s="8"/>
       <c r="E85" s="8" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="F85" s="8" t="s">
         <v>44</v>
       </c>
       <c r="G85" s="8" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H85" s="8" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="I85" s="8" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="J85" s="8"/>
       <c r="K85" s="7" t="s">
         <v>108</v>
       </c>
       <c r="L85" s="8" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="M85" s="9"/>
       <c r="N85" s="10"/>
@@ -5860,7 +5865,7 @@
     </row>
     <row r="86" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B86" s="7" t="n">
         <v>8</v>
@@ -5870,16 +5875,16 @@
       </c>
       <c r="D86" s="8"/>
       <c r="E86" s="8" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F86" s="8" t="s">
         <v>44</v>
       </c>
       <c r="G86" s="8" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="H86" s="8" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="I86" s="8"/>
       <c r="J86" s="8"/>
@@ -5895,7 +5900,7 @@
     </row>
     <row r="87" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B87" s="7" t="n">
         <v>8</v>
@@ -5905,16 +5910,16 @@
       </c>
       <c r="D87" s="8"/>
       <c r="E87" s="8" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="F87" s="8" t="s">
         <v>44</v>
       </c>
       <c r="G87" s="8" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="H87" s="8" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="I87" s="8"/>
       <c r="J87" s="8"/>
@@ -5930,7 +5935,7 @@
     </row>
     <row r="88" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B88" s="7" t="n">
         <v>8</v>
@@ -5942,26 +5947,26 @@
         <v>98</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F88" s="8" t="s">
         <v>44</v>
       </c>
       <c r="G88" s="8" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="H88" s="8" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="I88" s="8" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="J88" s="8"/>
       <c r="K88" s="7" t="s">
         <v>108</v>
       </c>
       <c r="L88" s="8" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="M88" s="9"/>
       <c r="N88" s="10"/>
@@ -5971,7 +5976,7 @@
     </row>
     <row r="89" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B89" s="7" t="n">
         <v>8</v>
@@ -5981,23 +5986,23 @@
       </c>
       <c r="D89" s="8"/>
       <c r="E89" s="8" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="F89" s="8" t="s">
         <v>44</v>
       </c>
       <c r="G89" s="8" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="H89" s="8" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="I89" s="8" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="J89" s="8"/>
       <c r="K89" s="7" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="L89" s="8"/>
       <c r="M89" s="9"/>
@@ -6008,7 +6013,7 @@
     </row>
     <row r="90" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B90" s="7" t="n">
         <v>8</v>
@@ -6018,7 +6023,7 @@
       </c>
       <c r="D90" s="8"/>
       <c r="E90" s="8" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="F90" s="8" t="s">
         <v>44</v>
@@ -6027,12 +6032,12 @@
         <v>89</v>
       </c>
       <c r="H90" s="8" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="I90" s="8"/>
       <c r="J90" s="8"/>
       <c r="K90" s="7" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="L90" s="8"/>
       <c r="M90" s="9"/>
@@ -6043,7 +6048,7 @@
     </row>
     <row r="91" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="7" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B91" s="7" t="n">
         <v>8</v>
@@ -6053,19 +6058,19 @@
       </c>
       <c r="D91" s="8"/>
       <c r="E91" s="8" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="F91" s="8" t="s">
         <v>44</v>
       </c>
       <c r="G91" s="8" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="H91" s="8" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="I91" s="8" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J91" s="8"/>
       <c r="K91" s="7" t="s">
@@ -6080,7 +6085,7 @@
     </row>
     <row r="92" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="7" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B92" s="7" t="n">
         <v>8</v>
@@ -6090,26 +6095,26 @@
       </c>
       <c r="D92" s="8"/>
       <c r="E92" s="8" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F92" s="8" t="s">
         <v>42</v>
       </c>
       <c r="G92" s="8" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="H92" s="8" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="I92" s="8"/>
       <c r="J92" s="8" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="K92" s="7" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="L92" s="8" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="M92" s="9"/>
       <c r="N92" s="10"/>
@@ -6119,7 +6124,7 @@
     </row>
     <row r="93" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="7" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B93" s="7" t="n">
         <v>8</v>
@@ -6129,7 +6134,7 @@
       </c>
       <c r="D93" s="8"/>
       <c r="E93" s="8" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="F93" s="8" t="s">
         <v>44</v>
@@ -6138,7 +6143,7 @@
         <v>89</v>
       </c>
       <c r="H93" s="8" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="I93" s="8"/>
       <c r="J93" s="8"/>
@@ -6154,7 +6159,7 @@
     </row>
     <row r="94" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="7" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B94" s="7" t="n">
         <v>8</v>
@@ -6164,16 +6169,16 @@
       </c>
       <c r="D94" s="8"/>
       <c r="E94" s="8" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="F94" s="8" t="s">
         <v>42</v>
       </c>
       <c r="G94" s="8" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="H94" s="8" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="I94" s="8" t="s">
         <v>79</v>
@@ -6233,25 +6238,25 @@
         <v>49</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="I1" s="6" t="s">
         <v>37</v>
@@ -6404,7 +6409,7 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13"/>
       <c r="B6" s="14" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C6" s="13" t="n">
         <f aca="false">SUM(C2:C5)</f>

</xml_diff>